<commit_message>
Cleaned and deleted all unwanted files and folders
</commit_message>
<xml_diff>
--- a/Documents/Freelance_Project_Template.xlsx
+++ b/Documents/Freelance_Project_Template.xlsx
@@ -16,9 +16,6 @@
     <sheet name="Component List" sheetId="2" r:id="rId2"/>
     <sheet name="Additional Project Information" sheetId="3" r:id="rId3"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Altimeter!$A$86:$F$105</definedName>
-  </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -40,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="149">
   <si>
     <t>M. Zaeem | Electronics &amp; Embedded Systems Engineer | BSc Electrical Engineering | MSc Autonomous Systems</t>
   </si>
@@ -394,9 +391,6 @@
     <t>Integrate sensors with MCU and implement non-volatile memory logging</t>
   </si>
   <si>
-    <t>Develop Python-based ground station interface for data retrieval via BLE</t>
-  </si>
-  <si>
     <t>Perform functional verification of sensor readout and data logging</t>
   </si>
   <si>
@@ -511,9 +505,6 @@
     <t>Backup Option Microcontroller for prototyping.</t>
   </si>
   <si>
-    <t>Pending</t>
-  </si>
-  <si>
     <t>Ordering PCBS</t>
   </si>
   <si>
@@ -526,7 +517,10 @@
     <t>Shipping to Client</t>
   </si>
   <si>
-    <t>In Progress</t>
+    <t>Not Needed</t>
+  </si>
+  <si>
+    <t>Develop Python-based ground station interface for data via BLE/Serial</t>
   </si>
 </sst>
 </file>
@@ -1555,18 +1549,10 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="18" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1574,6 +1560,120 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1583,6 +1683,102 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1601,22 +1797,13 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="15" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="15" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1641,210 +1828,17 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="20" fillId="5" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3677,82 +3671,82 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="158" t="s">
+      <c r="A1" s="188" t="s">
         <v>89</v>
       </c>
-      <c r="B1" s="159"/>
-      <c r="C1" s="159"/>
-      <c r="D1" s="159"/>
-      <c r="E1" s="159"/>
-      <c r="F1" s="160"/>
+      <c r="B1" s="189"/>
+      <c r="C1" s="189"/>
+      <c r="D1" s="189"/>
+      <c r="E1" s="189"/>
+      <c r="F1" s="190"/>
     </row>
     <row r="2" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="137" t="s">
+      <c r="A2" s="205" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="138"/>
-      <c r="C2" s="138"/>
-      <c r="D2" s="138"/>
-      <c r="E2" s="138"/>
-      <c r="F2" s="139"/>
+      <c r="B2" s="206"/>
+      <c r="C2" s="206"/>
+      <c r="D2" s="206"/>
+      <c r="E2" s="206"/>
+      <c r="F2" s="207"/>
     </row>
     <row r="3" spans="1:6" ht="4.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="137"/>
-      <c r="B3" s="138"/>
-      <c r="C3" s="138"/>
-      <c r="D3" s="138"/>
-      <c r="E3" s="138"/>
-      <c r="F3" s="139"/>
+      <c r="A3" s="205"/>
+      <c r="B3" s="206"/>
+      <c r="C3" s="206"/>
+      <c r="D3" s="206"/>
+      <c r="E3" s="206"/>
+      <c r="F3" s="207"/>
     </row>
     <row r="4" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="73" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="134"/>
-      <c r="C4" s="135"/>
-      <c r="D4" s="135"/>
-      <c r="E4" s="135"/>
-      <c r="F4" s="136"/>
+      <c r="B4" s="170"/>
+      <c r="C4" s="171"/>
+      <c r="D4" s="171"/>
+      <c r="E4" s="171"/>
+      <c r="F4" s="172"/>
     </row>
     <row r="5" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A5" s="33" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="168" t="s">
+      <c r="B5" s="199" t="s">
         <v>90</v>
       </c>
-      <c r="C5" s="168"/>
-      <c r="D5" s="168"/>
-      <c r="E5" s="168"/>
-      <c r="F5" s="169"/>
+      <c r="C5" s="199"/>
+      <c r="D5" s="199"/>
+      <c r="E5" s="199"/>
+      <c r="F5" s="200"/>
     </row>
     <row r="6" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A6" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="148" t="s">
+      <c r="B6" s="201" t="s">
         <v>88</v>
       </c>
-      <c r="C6" s="148"/>
-      <c r="D6" s="148"/>
-      <c r="E6" s="148"/>
-      <c r="F6" s="170"/>
+      <c r="C6" s="201"/>
+      <c r="D6" s="201"/>
+      <c r="E6" s="201"/>
+      <c r="F6" s="202"/>
     </row>
     <row r="7" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A7" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="147">
+      <c r="B7" s="213">
         <v>45929</v>
       </c>
-      <c r="C7" s="148"/>
+      <c r="C7" s="201"/>
       <c r="D7" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="E7" s="149">
-        <v>45961</v>
-      </c>
-      <c r="F7" s="150"/>
+      <c r="E7" s="214">
+        <v>46032</v>
+      </c>
+      <c r="F7" s="215"/>
     </row>
     <row r="8" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A8" s="43" t="s">
@@ -3764,21 +3758,21 @@
       <c r="C8" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="E8" s="151"/>
-      <c r="F8" s="152"/>
+      <c r="E8" s="216"/>
+      <c r="F8" s="217"/>
     </row>
     <row r="9" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A9" s="34" t="s">
         <v>9</v>
       </c>
-      <c r="B9" s="145">
+      <c r="B9" s="212">
         <v>15</v>
       </c>
-      <c r="C9" s="145"/>
-      <c r="D9" s="146" t="s">
+      <c r="C9" s="212"/>
+      <c r="D9" s="203" t="s">
         <v>10</v>
       </c>
-      <c r="E9" s="146"/>
+      <c r="E9" s="203"/>
       <c r="F9" s="95">
         <v>1500</v>
       </c>
@@ -3789,94 +3783,94 @@
       </c>
       <c r="B10" s="21"/>
       <c r="C10" s="22"/>
-      <c r="D10" s="146"/>
-      <c r="E10" s="146"/>
+      <c r="D10" s="203"/>
+      <c r="E10" s="203"/>
       <c r="F10" s="35"/>
     </row>
     <row r="11" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A11" s="140"/>
-      <c r="B11" s="141"/>
-      <c r="C11" s="141"/>
-      <c r="D11" s="141"/>
-      <c r="E11" s="141"/>
-      <c r="F11" s="142"/>
+      <c r="A11" s="208"/>
+      <c r="B11" s="209"/>
+      <c r="C11" s="209"/>
+      <c r="D11" s="209"/>
+      <c r="E11" s="209"/>
+      <c r="F11" s="210"/>
     </row>
     <row r="12" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="165" t="s">
+      <c r="A12" s="195" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="166"/>
-      <c r="C12" s="166"/>
-      <c r="D12" s="166"/>
-      <c r="E12" s="166"/>
-      <c r="F12" s="167"/>
+      <c r="B12" s="196"/>
+      <c r="C12" s="196"/>
+      <c r="D12" s="196"/>
+      <c r="E12" s="196"/>
+      <c r="F12" s="197"/>
     </row>
     <row r="13" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="161"/>
-      <c r="B13" s="162"/>
-      <c r="C13" s="162"/>
-      <c r="D13" s="162"/>
-      <c r="E13" s="162"/>
-      <c r="F13" s="163"/>
+      <c r="A13" s="191"/>
+      <c r="B13" s="192"/>
+      <c r="C13" s="192"/>
+      <c r="D13" s="192"/>
+      <c r="E13" s="192"/>
+      <c r="F13" s="193"/>
     </row>
     <row r="14" spans="1:6" ht="168" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="164"/>
-      <c r="B14" s="162"/>
-      <c r="C14" s="162"/>
-      <c r="D14" s="162"/>
-      <c r="E14" s="162"/>
-      <c r="F14" s="163"/>
+      <c r="A14" s="194"/>
+      <c r="B14" s="192"/>
+      <c r="C14" s="192"/>
+      <c r="D14" s="192"/>
+      <c r="E14" s="192"/>
+      <c r="F14" s="193"/>
     </row>
     <row r="15" spans="1:6" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="164"/>
-      <c r="B15" s="162"/>
-      <c r="C15" s="162"/>
-      <c r="D15" s="162"/>
-      <c r="E15" s="162"/>
-      <c r="F15" s="163"/>
+      <c r="A15" s="194"/>
+      <c r="B15" s="192"/>
+      <c r="C15" s="192"/>
+      <c r="D15" s="192"/>
+      <c r="E15" s="192"/>
+      <c r="F15" s="193"/>
     </row>
     <row r="16" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A16" s="164"/>
-      <c r="B16" s="162"/>
-      <c r="C16" s="162"/>
-      <c r="D16" s="162"/>
-      <c r="E16" s="162"/>
-      <c r="F16" s="163"/>
+      <c r="A16" s="194"/>
+      <c r="B16" s="192"/>
+      <c r="C16" s="192"/>
+      <c r="D16" s="192"/>
+      <c r="E16" s="192"/>
+      <c r="F16" s="193"/>
     </row>
     <row r="17" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A17" s="164"/>
-      <c r="B17" s="162"/>
-      <c r="C17" s="162"/>
-      <c r="D17" s="162"/>
-      <c r="E17" s="162"/>
-      <c r="F17" s="163"/>
+      <c r="A17" s="194"/>
+      <c r="B17" s="192"/>
+      <c r="C17" s="192"/>
+      <c r="D17" s="192"/>
+      <c r="E17" s="192"/>
+      <c r="F17" s="193"/>
     </row>
     <row r="18" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A18" s="164"/>
-      <c r="B18" s="162"/>
-      <c r="C18" s="162"/>
-      <c r="D18" s="162"/>
-      <c r="E18" s="162"/>
-      <c r="F18" s="163"/>
+      <c r="A18" s="194"/>
+      <c r="B18" s="192"/>
+      <c r="C18" s="192"/>
+      <c r="D18" s="192"/>
+      <c r="E18" s="192"/>
+      <c r="F18" s="193"/>
     </row>
     <row r="19" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" s="98" t="s">
         <v>13</v>
       </c>
-      <c r="B19" s="184"/>
-      <c r="C19" s="143"/>
+      <c r="B19" s="155"/>
+      <c r="C19" s="204"/>
       <c r="D19" s="97"/>
-      <c r="E19" s="143"/>
-      <c r="F19" s="144"/>
+      <c r="E19" s="204"/>
+      <c r="F19" s="211"/>
     </row>
     <row r="20" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A20" s="129" t="s">
-        <v>112</v>
-      </c>
-      <c r="B20" s="130" t="s">
+      <c r="A20" s="127" t="s">
+        <v>111</v>
+      </c>
+      <c r="B20" s="128" t="s">
         <v>15</v>
       </c>
-      <c r="C20" s="131"/>
+      <c r="C20" s="129"/>
       <c r="D20" s="5" t="s">
         <v>16</v>
       </c>
@@ -3888,98 +3882,98 @@
       </c>
     </row>
     <row r="21" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="129"/>
-      <c r="B21" s="132" t="s">
+      <c r="A21" s="127"/>
+      <c r="B21" s="130" t="s">
         <v>98</v>
       </c>
-      <c r="C21" s="133"/>
+      <c r="C21" s="131"/>
       <c r="D21" s="7">
         <v>6</v>
       </c>
-      <c r="E21" s="153" t="s">
-        <v>115</v>
+      <c r="E21" s="132" t="s">
+        <v>114</v>
       </c>
       <c r="F21" s="114" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A22" s="129"/>
-      <c r="B22" s="132" t="s">
+      <c r="A22" s="127"/>
+      <c r="B22" s="130" t="s">
         <v>99</v>
       </c>
-      <c r="C22" s="133"/>
+      <c r="C22" s="131"/>
       <c r="D22" s="8">
         <v>2</v>
       </c>
-      <c r="E22" s="154"/>
+      <c r="E22" s="133"/>
       <c r="F22" s="114" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A23" s="129"/>
-      <c r="B23" s="132" t="s">
+      <c r="A23" s="127"/>
+      <c r="B23" s="130" t="s">
         <v>100</v>
       </c>
-      <c r="C23" s="133"/>
+      <c r="C23" s="131"/>
       <c r="D23" s="8">
         <v>2</v>
       </c>
-      <c r="E23" s="154"/>
+      <c r="E23" s="133"/>
       <c r="F23" s="114" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A24" s="129"/>
-      <c r="B24" s="132" t="s">
+      <c r="A24" s="127"/>
+      <c r="B24" s="130" t="s">
         <v>101</v>
       </c>
-      <c r="C24" s="133"/>
+      <c r="C24" s="131"/>
       <c r="D24" s="8">
         <v>1</v>
       </c>
-      <c r="E24" s="154"/>
+      <c r="E24" s="133"/>
       <c r="F24" s="114" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A25" s="129"/>
-      <c r="B25" s="132" t="s">
+      <c r="A25" s="127"/>
+      <c r="B25" s="130" t="s">
         <v>102</v>
       </c>
-      <c r="C25" s="133"/>
+      <c r="C25" s="131"/>
       <c r="D25" s="9">
         <v>5</v>
       </c>
-      <c r="E25" s="154"/>
+      <c r="E25" s="133"/>
       <c r="F25" s="114" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A26" s="64"/>
-      <c r="B26" s="156" t="s">
+      <c r="B26" s="137" t="s">
         <v>19</v>
       </c>
-      <c r="C26" s="157"/>
+      <c r="C26" s="138"/>
       <c r="D26" s="74">
         <f>SUM(D21:D25)</f>
         <v>16</v>
       </c>
-      <c r="E26" s="155"/>
+      <c r="E26" s="198"/>
       <c r="F26" s="37"/>
     </row>
     <row r="27" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A27" s="129" t="s">
-        <v>113</v>
-      </c>
-      <c r="B27" s="130" t="s">
+      <c r="A27" s="127" t="s">
+        <v>112</v>
+      </c>
+      <c r="B27" s="128" t="s">
         <v>15</v>
       </c>
-      <c r="C27" s="131"/>
+      <c r="C27" s="129"/>
       <c r="D27" s="5" t="s">
         <v>16</v>
       </c>
@@ -3991,88 +3985,88 @@
       </c>
     </row>
     <row r="28" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A28" s="129"/>
-      <c r="B28" s="132" t="s">
+      <c r="A28" s="127"/>
+      <c r="B28" s="130" t="s">
         <v>104</v>
       </c>
-      <c r="C28" s="133"/>
+      <c r="C28" s="131"/>
       <c r="D28" s="7">
         <v>26</v>
       </c>
-      <c r="E28" s="153" t="s">
+      <c r="E28" s="132" t="s">
         <v>103</v>
       </c>
       <c r="F28" s="114" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A29" s="129"/>
-      <c r="B29" s="132" t="s">
+      <c r="A29" s="127"/>
+      <c r="B29" s="130" t="s">
+        <v>148</v>
+      </c>
+      <c r="C29" s="131"/>
+      <c r="D29" s="8">
+        <v>18</v>
+      </c>
+      <c r="E29" s="133"/>
+      <c r="F29" s="114" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A30" s="127"/>
+      <c r="B30" s="130" t="s">
         <v>105</v>
       </c>
-      <c r="C29" s="133"/>
-      <c r="D29" s="8">
-        <v>16</v>
-      </c>
-      <c r="E29" s="154"/>
-      <c r="F29" s="114" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A30" s="129"/>
-      <c r="B30" s="132" t="s">
-        <v>106</v>
-      </c>
-      <c r="C30" s="133"/>
+      <c r="C30" s="131"/>
       <c r="D30" s="8">
         <v>4</v>
       </c>
-      <c r="E30" s="154"/>
+      <c r="E30" s="133"/>
       <c r="F30" s="114" t="s">
-        <v>149</v>
+        <v>122</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A31" s="129"/>
-      <c r="B31" s="132" t="s">
+      <c r="A31" s="127"/>
+      <c r="B31" s="130" t="s">
+        <v>106</v>
+      </c>
+      <c r="C31" s="131"/>
+      <c r="D31" s="8">
+        <v>2</v>
+      </c>
+      <c r="E31" s="133"/>
+      <c r="F31" s="114" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A32" s="127"/>
+      <c r="B32" s="130" t="s">
         <v>107</v>
       </c>
-      <c r="C31" s="133"/>
-      <c r="D31" s="8">
-        <v>4</v>
-      </c>
-      <c r="E31" s="154"/>
-      <c r="F31" s="114" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A32" s="129"/>
-      <c r="B32" s="132" t="s">
-        <v>108</v>
-      </c>
-      <c r="C32" s="133"/>
+      <c r="C32" s="131"/>
       <c r="D32" s="9">
-        <v>4</v>
-      </c>
-      <c r="E32" s="154"/>
+        <v>2</v>
+      </c>
+      <c r="E32" s="133"/>
       <c r="F32" s="114" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A33" s="64"/>
-      <c r="B33" s="156" t="s">
+      <c r="B33" s="137" t="s">
         <v>21</v>
       </c>
-      <c r="C33" s="157"/>
+      <c r="C33" s="138"/>
       <c r="D33" s="74">
         <f>SUM(D28:D32)</f>
-        <v>54</v>
-      </c>
-      <c r="E33" s="155"/>
+        <v>52</v>
+      </c>
+      <c r="E33" s="198"/>
       <c r="F33" s="37"/>
     </row>
     <row r="34" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
@@ -4084,13 +4078,13 @@
       <c r="F34" s="37"/>
     </row>
     <row r="35" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A35" s="129" t="s">
-        <v>114</v>
-      </c>
-      <c r="B35" s="130" t="s">
+      <c r="A35" s="127" t="s">
+        <v>113</v>
+      </c>
+      <c r="B35" s="128" t="s">
         <v>15</v>
       </c>
-      <c r="C35" s="131"/>
+      <c r="C35" s="129"/>
       <c r="D35" s="5" t="s">
         <v>16</v>
       </c>
@@ -4102,127 +4096,139 @@
       </c>
     </row>
     <row r="36" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A36" s="129"/>
-      <c r="B36" s="132" t="s">
-        <v>110</v>
-      </c>
-      <c r="C36" s="133"/>
+      <c r="A36" s="127"/>
+      <c r="B36" s="130" t="s">
+        <v>109</v>
+      </c>
+      <c r="C36" s="131"/>
       <c r="D36" s="7">
         <v>16</v>
       </c>
-      <c r="E36" s="153" t="s">
-        <v>116</v>
+      <c r="E36" s="132" t="s">
+        <v>115</v>
       </c>
       <c r="F36" s="114" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A37" s="129"/>
-      <c r="B37" s="132" t="s">
-        <v>109</v>
-      </c>
-      <c r="C37" s="133"/>
-      <c r="D37" s="8"/>
-      <c r="E37" s="154"/>
+      <c r="A37" s="127"/>
+      <c r="B37" s="130" t="s">
+        <v>108</v>
+      </c>
+      <c r="C37" s="131"/>
+      <c r="D37" s="8">
+        <v>8</v>
+      </c>
+      <c r="E37" s="133"/>
       <c r="F37" s="114" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A38" s="127"/>
+      <c r="B38" s="130" t="s">
+        <v>110</v>
+      </c>
+      <c r="C38" s="131"/>
+      <c r="D38" s="8">
+        <v>5</v>
+      </c>
+      <c r="E38" s="133"/>
+      <c r="F38" s="114" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A39" s="127"/>
+      <c r="B39" s="130" t="s">
+        <v>143</v>
+      </c>
+      <c r="C39" s="131"/>
+      <c r="D39" s="8">
+        <v>0</v>
+      </c>
+      <c r="E39" s="133"/>
+      <c r="F39" s="114" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A40" s="127"/>
+      <c r="B40" s="130" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A38" s="129"/>
-      <c r="B38" s="132" t="s">
-        <v>111</v>
-      </c>
-      <c r="C38" s="133"/>
-      <c r="D38" s="8"/>
-      <c r="E38" s="154"/>
-      <c r="F38" s="114" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A39" s="129"/>
-      <c r="B39" s="132" t="s">
+      <c r="C40" s="131"/>
+      <c r="D40" s="8">
+        <v>0</v>
+      </c>
+      <c r="E40" s="133"/>
+      <c r="F40" s="114" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A41" s="127"/>
+      <c r="B41" s="218" t="s">
         <v>145</v>
       </c>
-      <c r="C39" s="133"/>
-      <c r="D39" s="8"/>
-      <c r="E39" s="154"/>
-      <c r="F39" s="114" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A40" s="129"/>
-      <c r="B40" s="132" t="s">
+      <c r="C41" s="219"/>
+      <c r="D41" s="8">
+        <v>0</v>
+      </c>
+      <c r="E41" s="133"/>
+      <c r="F41" s="114" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="14.45" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="127"/>
+      <c r="B42" s="220" t="s">
         <v>146</v>
       </c>
-      <c r="C40" s="133"/>
-      <c r="D40" s="9"/>
-      <c r="E40" s="154"/>
-      <c r="F40" s="114" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A41" s="129"/>
-      <c r="B41" s="125" t="s">
+      <c r="C42" s="221"/>
+      <c r="D42" s="8">
+        <v>0</v>
+      </c>
+      <c r="E42" s="133"/>
+      <c r="F42" s="114" t="s">
         <v>147</v>
-      </c>
-      <c r="C41" s="126"/>
-      <c r="D41" s="9"/>
-      <c r="E41" s="154"/>
-      <c r="F41" s="114" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" ht="14.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="129"/>
-      <c r="B42" s="127" t="s">
-        <v>148</v>
-      </c>
-      <c r="C42" s="128"/>
-      <c r="D42" s="9"/>
-      <c r="E42" s="154"/>
-      <c r="F42" s="114" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A43" s="64"/>
-      <c r="B43" s="156" t="s">
+      <c r="B43" s="137" t="s">
         <v>23</v>
       </c>
-      <c r="C43" s="157"/>
+      <c r="C43" s="138"/>
       <c r="D43" s="74">
         <f>SUM(D36:D42)</f>
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="E43" s="63"/>
       <c r="F43" s="75"/>
     </row>
     <row r="44" spans="1:6" s="2" customFormat="1" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A44" s="216"/>
-      <c r="B44" s="217"/>
-      <c r="C44" s="217"/>
-      <c r="D44" s="217"/>
-      <c r="E44" s="217"/>
-      <c r="F44" s="218"/>
+      <c r="A44" s="134"/>
+      <c r="B44" s="135"/>
+      <c r="C44" s="135"/>
+      <c r="D44" s="135"/>
+      <c r="E44" s="135"/>
+      <c r="F44" s="136"/>
     </row>
     <row r="45" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="183" t="s">
+      <c r="A45" s="154" t="s">
         <v>24</v>
       </c>
-      <c r="B45" s="184"/>
+      <c r="B45" s="155"/>
       <c r="C45" s="76" t="s">
         <v>25</v>
       </c>
-      <c r="D45" s="134" t="s">
+      <c r="D45" s="170" t="s">
         <v>26</v>
       </c>
-      <c r="E45" s="135"/>
-      <c r="F45" s="136"/>
+      <c r="E45" s="171"/>
+      <c r="F45" s="172"/>
     </row>
     <row r="46" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A46" s="39" t="s">
@@ -4232,11 +4238,11 @@
       <c r="C46" s="99" t="s">
         <v>28</v>
       </c>
-      <c r="D46" s="199" t="s">
+      <c r="D46" s="173" t="s">
         <v>29</v>
       </c>
-      <c r="E46" s="200"/>
-      <c r="F46" s="201"/>
+      <c r="E46" s="174"/>
+      <c r="F46" s="175"/>
     </row>
     <row r="47" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A47" s="39" t="s">
@@ -4246,9 +4252,9 @@
       <c r="C47" s="100" t="s">
         <v>92</v>
       </c>
-      <c r="D47" s="202"/>
-      <c r="E47" s="203"/>
-      <c r="F47" s="204"/>
+      <c r="D47" s="176"/>
+      <c r="E47" s="177"/>
+      <c r="F47" s="178"/>
     </row>
     <row r="48" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A48" s="39" t="s">
@@ -4258,9 +4264,9 @@
       <c r="C48" s="100" t="s">
         <v>91</v>
       </c>
-      <c r="D48" s="202"/>
-      <c r="E48" s="203"/>
-      <c r="F48" s="204"/>
+      <c r="D48" s="176"/>
+      <c r="E48" s="177"/>
+      <c r="F48" s="178"/>
     </row>
     <row r="49" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A49" s="39" t="s">
@@ -4270,9 +4276,9 @@
       <c r="C49" s="100" t="s">
         <v>93</v>
       </c>
-      <c r="D49" s="202"/>
-      <c r="E49" s="203"/>
-      <c r="F49" s="204"/>
+      <c r="D49" s="176"/>
+      <c r="E49" s="177"/>
+      <c r="F49" s="178"/>
     </row>
     <row r="50" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A50" s="39" t="s">
@@ -4282,9 +4288,9 @@
       <c r="C50" s="100" t="s">
         <v>94</v>
       </c>
-      <c r="D50" s="205"/>
-      <c r="E50" s="206"/>
-      <c r="F50" s="207"/>
+      <c r="D50" s="179"/>
+      <c r="E50" s="180"/>
+      <c r="F50" s="181"/>
     </row>
     <row r="51" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A51" s="39" t="s">
@@ -4294,11 +4300,11 @@
       <c r="C51" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="D51" s="191" t="s">
+      <c r="D51" s="162" t="s">
         <v>36</v>
       </c>
-      <c r="E51" s="192"/>
-      <c r="F51" s="193"/>
+      <c r="E51" s="163"/>
+      <c r="F51" s="164"/>
     </row>
     <row r="52" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A52" s="39" t="s">
@@ -4308,11 +4314,11 @@
       <c r="C52" s="49" t="s">
         <v>95</v>
       </c>
-      <c r="D52" s="194" t="s">
+      <c r="D52" s="165" t="s">
         <v>38</v>
       </c>
-      <c r="E52" s="195"/>
-      <c r="F52" s="196"/>
+      <c r="E52" s="166"/>
+      <c r="F52" s="167"/>
     </row>
     <row r="53" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A53" s="39" t="s">
@@ -4322,11 +4328,11 @@
       <c r="C53" s="49" t="s">
         <v>96</v>
       </c>
-      <c r="D53" s="194" t="s">
+      <c r="D53" s="165" t="s">
         <v>40</v>
       </c>
-      <c r="E53" s="195"/>
-      <c r="F53" s="196"/>
+      <c r="E53" s="166"/>
+      <c r="F53" s="167"/>
     </row>
     <row r="54" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A54" s="39" t="s">
@@ -4336,11 +4342,11 @@
       <c r="C54" s="49" t="s">
         <v>97</v>
       </c>
-      <c r="D54" s="194" t="s">
+      <c r="D54" s="165" t="s">
         <v>42</v>
       </c>
-      <c r="E54" s="195"/>
-      <c r="F54" s="196"/>
+      <c r="E54" s="166"/>
+      <c r="F54" s="167"/>
     </row>
     <row r="55" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A55" s="39" t="s">
@@ -4348,78 +4354,78 @@
       </c>
       <c r="B55" s="50"/>
       <c r="C55" s="49"/>
-      <c r="D55" s="194" t="s">
+      <c r="D55" s="165" t="s">
         <v>44</v>
       </c>
-      <c r="E55" s="195"/>
-      <c r="F55" s="196"/>
+      <c r="E55" s="166"/>
+      <c r="F55" s="167"/>
     </row>
     <row r="56" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A56" s="219"/>
-      <c r="B56" s="220"/>
-      <c r="C56" s="220"/>
-      <c r="D56" s="220"/>
-      <c r="E56" s="220"/>
-      <c r="F56" s="221"/>
+      <c r="A56" s="139"/>
+      <c r="B56" s="140"/>
+      <c r="C56" s="140"/>
+      <c r="D56" s="140"/>
+      <c r="E56" s="140"/>
+      <c r="F56" s="141"/>
     </row>
     <row r="57" spans="1:6" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A57" s="188" t="s">
+      <c r="A57" s="159" t="s">
         <v>76</v>
       </c>
-      <c r="B57" s="197"/>
-      <c r="C57" s="197"/>
-      <c r="D57" s="197"/>
-      <c r="E57" s="197"/>
-      <c r="F57" s="198"/>
+      <c r="B57" s="168"/>
+      <c r="C57" s="168"/>
+      <c r="D57" s="168"/>
+      <c r="E57" s="168"/>
+      <c r="F57" s="169"/>
     </row>
     <row r="58" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A58" s="215" t="s">
+      <c r="A58" s="125" t="s">
         <v>45</v>
       </c>
-      <c r="B58" s="215"/>
-      <c r="C58" s="215"/>
-      <c r="D58" s="215"/>
-      <c r="E58" s="215"/>
+      <c r="B58" s="125"/>
+      <c r="C58" s="125"/>
+      <c r="D58" s="125"/>
+      <c r="E58" s="125"/>
       <c r="F58" s="96" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="59" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A59" s="211"/>
-      <c r="B59" s="211"/>
-      <c r="C59" s="211"/>
-      <c r="D59" s="211"/>
-      <c r="E59" s="211"/>
+      <c r="A59" s="126"/>
+      <c r="B59" s="126"/>
+      <c r="C59" s="126"/>
+      <c r="D59" s="126"/>
+      <c r="E59" s="126"/>
       <c r="F59" s="57"/>
     </row>
     <row r="60" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A60" s="211"/>
-      <c r="B60" s="211"/>
-      <c r="C60" s="211"/>
-      <c r="D60" s="211"/>
-      <c r="E60" s="211"/>
+      <c r="A60" s="126"/>
+      <c r="B60" s="126"/>
+      <c r="C60" s="126"/>
+      <c r="D60" s="126"/>
+      <c r="E60" s="126"/>
       <c r="F60" s="58"/>
     </row>
     <row r="61" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A61" s="77"/>
       <c r="B61" s="78"/>
-      <c r="C61" s="212" t="s">
+      <c r="C61" s="185" t="s">
         <v>73</v>
       </c>
-      <c r="D61" s="213"/>
-      <c r="E61" s="214"/>
+      <c r="D61" s="186"/>
+      <c r="E61" s="187"/>
       <c r="F61" s="79">
         <f>SUM(F59:F60)</f>
         <v>0</v>
       </c>
     </row>
     <row r="62" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A62" s="208"/>
-      <c r="B62" s="209"/>
-      <c r="C62" s="209"/>
-      <c r="D62" s="209"/>
-      <c r="E62" s="209"/>
-      <c r="F62" s="210"/>
+      <c r="A62" s="182"/>
+      <c r="B62" s="183"/>
+      <c r="C62" s="183"/>
+      <c r="D62" s="183"/>
+      <c r="E62" s="183"/>
+      <c r="F62" s="184"/>
     </row>
     <row r="63" spans="1:6" s="3" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="66" t="s">
@@ -4442,13 +4448,13 @@
         <v>54</v>
       </c>
       <c r="D64" s="25" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E64" s="26" t="s">
         <v>55</v>
       </c>
       <c r="F64" s="45" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="65" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
@@ -4583,51 +4589,51 @@
       </c>
     </row>
     <row r="74" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A74" s="171"/>
-      <c r="B74" s="172"/>
-      <c r="C74" s="172"/>
-      <c r="D74" s="172"/>
-      <c r="E74" s="172"/>
-      <c r="F74" s="173"/>
+      <c r="A74" s="142"/>
+      <c r="B74" s="143"/>
+      <c r="C74" s="143"/>
+      <c r="D74" s="143"/>
+      <c r="E74" s="143"/>
+      <c r="F74" s="144"/>
     </row>
     <row r="75" spans="1:7" s="3" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A75" s="188" t="s">
+      <c r="A75" s="159" t="s">
         <v>78</v>
       </c>
-      <c r="B75" s="189"/>
-      <c r="C75" s="189"/>
-      <c r="D75" s="189"/>
-      <c r="E75" s="189"/>
-      <c r="F75" s="190"/>
+      <c r="B75" s="160"/>
+      <c r="C75" s="160"/>
+      <c r="D75" s="160"/>
+      <c r="E75" s="160"/>
+      <c r="F75" s="161"/>
     </row>
     <row r="76" spans="1:7" s="3" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A76" s="185" t="s">
+      <c r="A76" s="156" t="s">
         <v>46</v>
       </c>
-      <c r="B76" s="186"/>
-      <c r="C76" s="186"/>
-      <c r="D76" s="186"/>
-      <c r="E76" s="186"/>
-      <c r="F76" s="187"/>
+      <c r="B76" s="157"/>
+      <c r="C76" s="157"/>
+      <c r="D76" s="157"/>
+      <c r="E76" s="157"/>
+      <c r="F76" s="158"/>
     </row>
     <row r="77" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A77" s="40" t="s">
         <v>47</v>
       </c>
       <c r="B77" s="14" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C77" s="13" t="s">
         <v>48</v>
       </c>
       <c r="D77" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="E77" s="16" t="s">
+        <v>120</v>
+      </c>
+      <c r="F77" s="41" t="s">
         <v>119</v>
-      </c>
-      <c r="E77" s="16" t="s">
-        <v>121</v>
-      </c>
-      <c r="F77" s="41" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="78" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
@@ -4664,18 +4670,18 @@
       </c>
       <c r="C79" s="51">
         <f>D33</f>
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D79" s="108">
         <f t="shared" ref="D79:D81" si="1">B79*C79</f>
-        <v>810</v>
+        <v>780</v>
       </c>
       <c r="E79" s="109">
-        <v>429</v>
+        <v>858</v>
       </c>
       <c r="F79" s="104">
         <f t="shared" ref="F79:F82" si="2">D79-E79</f>
-        <v>381</v>
+        <v>-78</v>
       </c>
       <c r="G79" s="4"/>
     </row>
@@ -4689,18 +4695,18 @@
       </c>
       <c r="C80" s="54">
         <f>D43</f>
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="D80" s="110">
         <f t="shared" si="1"/>
-        <v>240</v>
+        <v>435</v>
       </c>
       <c r="E80" s="109">
         <v>429</v>
       </c>
       <c r="F80" s="105">
         <f t="shared" si="2"/>
-        <v>-189</v>
+        <v>6</v>
       </c>
     </row>
     <row r="81" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -4719,9 +4725,9 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="E81" s="106"/>
+      <c r="E81" s="109"/>
       <c r="F81" s="106">
-        <f t="shared" si="2"/>
+        <f>D81-E81</f>
         <v>0</v>
       </c>
     </row>
@@ -4752,19 +4758,19 @@
       <c r="B83" s="80"/>
       <c r="C83" s="81">
         <f>SUM(C78:C81)</f>
-        <v>86</v>
+        <v>97</v>
       </c>
       <c r="D83" s="107">
         <f>SUM(D78:D82)</f>
-        <v>1290</v>
+        <v>1455</v>
       </c>
       <c r="E83" s="107">
         <f>SUM(E78:E81)</f>
-        <v>1029</v>
+        <v>1458</v>
       </c>
       <c r="F83" s="107">
         <f>SUM(F78:F82)</f>
-        <v>261</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="84" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -4784,182 +4790,203 @@
       <c r="F85" s="124"/>
     </row>
     <row r="86" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A86" s="174" t="s">
+      <c r="A86" s="145" t="s">
         <v>51</v>
       </c>
-      <c r="B86" s="175"/>
-      <c r="C86" s="175"/>
-      <c r="D86" s="175"/>
-      <c r="E86" s="175"/>
-      <c r="F86" s="176"/>
+      <c r="B86" s="146"/>
+      <c r="C86" s="146"/>
+      <c r="D86" s="146"/>
+      <c r="E86" s="146"/>
+      <c r="F86" s="147"/>
     </row>
     <row r="87" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A87" s="177"/>
-      <c r="B87" s="178"/>
-      <c r="C87" s="178"/>
-      <c r="D87" s="178"/>
-      <c r="E87" s="178"/>
-      <c r="F87" s="179"/>
+      <c r="A87" s="148"/>
+      <c r="B87" s="149"/>
+      <c r="C87" s="149"/>
+      <c r="D87" s="149"/>
+      <c r="E87" s="149"/>
+      <c r="F87" s="150"/>
     </row>
     <row r="88" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A88" s="177"/>
-      <c r="B88" s="178"/>
-      <c r="C88" s="178"/>
-      <c r="D88" s="178"/>
-      <c r="E88" s="178"/>
-      <c r="F88" s="179"/>
+      <c r="A88" s="148"/>
+      <c r="B88" s="149"/>
+      <c r="C88" s="149"/>
+      <c r="D88" s="149"/>
+      <c r="E88" s="149"/>
+      <c r="F88" s="150"/>
     </row>
     <row r="89" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A89" s="177"/>
-      <c r="B89" s="178"/>
-      <c r="C89" s="178"/>
-      <c r="D89" s="178"/>
-      <c r="E89" s="178"/>
-      <c r="F89" s="179"/>
+      <c r="A89" s="148"/>
+      <c r="B89" s="149"/>
+      <c r="C89" s="149"/>
+      <c r="D89" s="149"/>
+      <c r="E89" s="149"/>
+      <c r="F89" s="150"/>
     </row>
     <row r="90" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A90" s="177"/>
-      <c r="B90" s="178"/>
-      <c r="C90" s="178"/>
-      <c r="D90" s="178"/>
-      <c r="E90" s="178"/>
-      <c r="F90" s="179"/>
+      <c r="A90" s="148"/>
+      <c r="B90" s="149"/>
+      <c r="C90" s="149"/>
+      <c r="D90" s="149"/>
+      <c r="E90" s="149"/>
+      <c r="F90" s="150"/>
     </row>
     <row r="91" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A91" s="177"/>
-      <c r="B91" s="178"/>
-      <c r="C91" s="178"/>
-      <c r="D91" s="178"/>
-      <c r="E91" s="178"/>
-      <c r="F91" s="179"/>
+      <c r="A91" s="148"/>
+      <c r="B91" s="149"/>
+      <c r="C91" s="149"/>
+      <c r="D91" s="149"/>
+      <c r="E91" s="149"/>
+      <c r="F91" s="150"/>
     </row>
     <row r="92" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A92" s="177"/>
-      <c r="B92" s="178"/>
-      <c r="C92" s="178"/>
-      <c r="D92" s="178"/>
-      <c r="E92" s="178"/>
-      <c r="F92" s="179"/>
+      <c r="A92" s="148"/>
+      <c r="B92" s="149"/>
+      <c r="C92" s="149"/>
+      <c r="D92" s="149"/>
+      <c r="E92" s="149"/>
+      <c r="F92" s="150"/>
     </row>
     <row r="93" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A93" s="177"/>
-      <c r="B93" s="178"/>
-      <c r="C93" s="178"/>
-      <c r="D93" s="178"/>
-      <c r="E93" s="178"/>
-      <c r="F93" s="179"/>
+      <c r="A93" s="148"/>
+      <c r="B93" s="149"/>
+      <c r="C93" s="149"/>
+      <c r="D93" s="149"/>
+      <c r="E93" s="149"/>
+      <c r="F93" s="150"/>
     </row>
     <row r="94" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A94" s="177"/>
-      <c r="B94" s="178"/>
-      <c r="C94" s="178"/>
-      <c r="D94" s="178"/>
-      <c r="E94" s="178"/>
-      <c r="F94" s="179"/>
+      <c r="A94" s="148"/>
+      <c r="B94" s="149"/>
+      <c r="C94" s="149"/>
+      <c r="D94" s="149"/>
+      <c r="E94" s="149"/>
+      <c r="F94" s="150"/>
     </row>
     <row r="95" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A95" s="177"/>
-      <c r="B95" s="178"/>
-      <c r="C95" s="178"/>
-      <c r="D95" s="178"/>
-      <c r="E95" s="178"/>
-      <c r="F95" s="179"/>
+      <c r="A95" s="148"/>
+      <c r="B95" s="149"/>
+      <c r="C95" s="149"/>
+      <c r="D95" s="149"/>
+      <c r="E95" s="149"/>
+      <c r="F95" s="150"/>
     </row>
     <row r="96" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A96" s="177"/>
-      <c r="B96" s="178"/>
-      <c r="C96" s="178"/>
-      <c r="D96" s="178"/>
-      <c r="E96" s="178"/>
-      <c r="F96" s="179"/>
+      <c r="A96" s="148"/>
+      <c r="B96" s="149"/>
+      <c r="C96" s="149"/>
+      <c r="D96" s="149"/>
+      <c r="E96" s="149"/>
+      <c r="F96" s="150"/>
     </row>
     <row r="97" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A97" s="177"/>
-      <c r="B97" s="178"/>
-      <c r="C97" s="178"/>
-      <c r="D97" s="178"/>
-      <c r="E97" s="178"/>
-      <c r="F97" s="179"/>
+      <c r="A97" s="148"/>
+      <c r="B97" s="149"/>
+      <c r="C97" s="149"/>
+      <c r="D97" s="149"/>
+      <c r="E97" s="149"/>
+      <c r="F97" s="150"/>
     </row>
     <row r="98" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A98" s="177"/>
-      <c r="B98" s="178"/>
-      <c r="C98" s="178"/>
-      <c r="D98" s="178"/>
-      <c r="E98" s="178"/>
-      <c r="F98" s="179"/>
+      <c r="A98" s="148"/>
+      <c r="B98" s="149"/>
+      <c r="C98" s="149"/>
+      <c r="D98" s="149"/>
+      <c r="E98" s="149"/>
+      <c r="F98" s="150"/>
     </row>
     <row r="99" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A99" s="177"/>
-      <c r="B99" s="178"/>
-      <c r="C99" s="178"/>
-      <c r="D99" s="178"/>
-      <c r="E99" s="178"/>
-      <c r="F99" s="179"/>
+      <c r="A99" s="148"/>
+      <c r="B99" s="149"/>
+      <c r="C99" s="149"/>
+      <c r="D99" s="149"/>
+      <c r="E99" s="149"/>
+      <c r="F99" s="150"/>
     </row>
     <row r="100" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A100" s="177"/>
-      <c r="B100" s="178"/>
-      <c r="C100" s="178"/>
-      <c r="D100" s="178"/>
-      <c r="E100" s="178"/>
-      <c r="F100" s="179"/>
+      <c r="A100" s="148"/>
+      <c r="B100" s="149"/>
+      <c r="C100" s="149"/>
+      <c r="D100" s="149"/>
+      <c r="E100" s="149"/>
+      <c r="F100" s="150"/>
     </row>
     <row r="101" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A101" s="177"/>
-      <c r="B101" s="178"/>
-      <c r="C101" s="178"/>
-      <c r="D101" s="178"/>
-      <c r="E101" s="178"/>
-      <c r="F101" s="179"/>
+      <c r="A101" s="148"/>
+      <c r="B101" s="149"/>
+      <c r="C101" s="149"/>
+      <c r="D101" s="149"/>
+      <c r="E101" s="149"/>
+      <c r="F101" s="150"/>
     </row>
     <row r="102" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A102" s="177"/>
-      <c r="B102" s="178"/>
-      <c r="C102" s="178"/>
-      <c r="D102" s="178"/>
-      <c r="E102" s="178"/>
-      <c r="F102" s="179"/>
+      <c r="A102" s="148"/>
+      <c r="B102" s="149"/>
+      <c r="C102" s="149"/>
+      <c r="D102" s="149"/>
+      <c r="E102" s="149"/>
+      <c r="F102" s="150"/>
     </row>
     <row r="103" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A103" s="177"/>
-      <c r="B103" s="178"/>
-      <c r="C103" s="178"/>
-      <c r="D103" s="178"/>
-      <c r="E103" s="178"/>
-      <c r="F103" s="179"/>
+      <c r="A103" s="148"/>
+      <c r="B103" s="149"/>
+      <c r="C103" s="149"/>
+      <c r="D103" s="149"/>
+      <c r="E103" s="149"/>
+      <c r="F103" s="150"/>
     </row>
     <row r="104" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A104" s="177"/>
-      <c r="B104" s="178"/>
-      <c r="C104" s="178"/>
-      <c r="D104" s="178"/>
-      <c r="E104" s="178"/>
-      <c r="F104" s="179"/>
+      <c r="A104" s="148"/>
+      <c r="B104" s="149"/>
+      <c r="C104" s="149"/>
+      <c r="D104" s="149"/>
+      <c r="E104" s="149"/>
+      <c r="F104" s="150"/>
     </row>
     <row r="105" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A105" s="180"/>
-      <c r="B105" s="181"/>
-      <c r="C105" s="181"/>
-      <c r="D105" s="181"/>
-      <c r="E105" s="181"/>
-      <c r="F105" s="182"/>
+      <c r="A105" s="151"/>
+      <c r="B105" s="152"/>
+      <c r="C105" s="152"/>
+      <c r="D105" s="152"/>
+      <c r="E105" s="152"/>
+      <c r="F105" s="153"/>
     </row>
   </sheetData>
   <mergeCells count="65">
-    <mergeCell ref="A58:E58"/>
-    <mergeCell ref="A59:E59"/>
-    <mergeCell ref="A35:A42"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="E36:E42"/>
-    <mergeCell ref="A44:F44"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="B43:C43"/>
-    <mergeCell ref="A56:F56"/>
+    <mergeCell ref="A27:A32"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="A2:F3"/>
+    <mergeCell ref="A20:A25"/>
+    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="E28:E33"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A13:F18"/>
+    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="E21:E26"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B4:F4"/>
     <mergeCell ref="A74:F74"/>
     <mergeCell ref="A86:F105"/>
     <mergeCell ref="A45:B45"/>
@@ -4976,42 +5003,21 @@
     <mergeCell ref="A62:F62"/>
     <mergeCell ref="A60:E60"/>
     <mergeCell ref="C61:E61"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A13:F18"/>
-    <mergeCell ref="A12:F12"/>
-    <mergeCell ref="E21:E26"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B5:F5"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="E28:E33"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="A2:F3"/>
-    <mergeCell ref="A20:A25"/>
-    <mergeCell ref="A11:F11"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="A58:E58"/>
+    <mergeCell ref="A59:E59"/>
+    <mergeCell ref="A35:A42"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="E36:E42"/>
+    <mergeCell ref="A44:F44"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="B43:C43"/>
+    <mergeCell ref="A56:F56"/>
     <mergeCell ref="B41:C41"/>
     <mergeCell ref="B42:C42"/>
-    <mergeCell ref="A27:A32"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B28:C28"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="60" fitToHeight="0" orientation="portrait" r:id="rId1"/>
@@ -5346,16 +5352,16 @@
         <v>80</v>
       </c>
       <c r="E1" s="117" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F1" s="88" t="s">
         <v>81</v>
       </c>
       <c r="G1" s="119" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="H1" s="93" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I1" s="59"/>
       <c r="J1" s="59"/>
@@ -5366,16 +5372,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="91" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C2" s="85" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D2" s="85" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E2" s="92" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F2" s="86">
         <v>1</v>
@@ -5396,16 +5402,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="86" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C3" s="85" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D3" s="85" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E3" s="92" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F3" s="86">
         <v>1</v>
@@ -5426,16 +5432,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="86" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C4" s="85" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D4" s="85" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E4" s="92" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F4" s="86">
         <v>1</v>
@@ -5456,16 +5462,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="91" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C5" s="85" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D5" s="85" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E5" s="92" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F5" s="86">
         <v>1</v>
@@ -5486,16 +5492,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="120" t="s">
+        <v>141</v>
+      </c>
+      <c r="C6" s="121" t="s">
+        <v>140</v>
+      </c>
+      <c r="D6" s="85" t="s">
         <v>142</v>
       </c>
-      <c r="C6" s="121" t="s">
-        <v>141</v>
-      </c>
-      <c r="D6" s="85" t="s">
-        <v>143</v>
-      </c>
       <c r="E6" s="92" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F6" s="86">
         <v>1</v>
@@ -5873,7 +5879,7 @@
   <sheetData>
     <row r="1" spans="1:9" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A1" s="224" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B1" s="224"/>
       <c r="C1" s="224"/>

</xml_diff>